<commit_message>
Acerta limite dos dias da senha
</commit_message>
<xml_diff>
--- a/estagiarios.xlsx
+++ b/estagiarios.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="62">
   <si>
     <t xml:space="preserve">NOME</t>
   </si>
@@ -131,6 +131,81 @@
   </si>
   <si>
     <t xml:space="preserve">Posto de Identificação Civil de Colatina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alexsandra Victoria dos Santos Jesus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posto de Identificação Civil de Serra Sede</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5170915</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brenno de Jesus Coelho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posto de Identificação Civil de Via Velha - Boulevard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezequiel Lupe Azevedo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posto de Identificação Civil de Cachoeiro de Itapemirim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heloa Medeiros Ramos dos Santos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">João Gabriel Alves Correia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posto de Identificação Civil da ALes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAUA KELVIN MOREIRA SOARES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posto de Identificação Civil de Vila Velha - Boulevard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luiza Nicholle Siqueira Bezerra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lyandra Machado Zanelato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posto de Identificação Civil de Linhares</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCELA BORGES DA SILVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maria Clara Leal Lorenconis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARIANY DE SANTANA DOS SANTOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARINA FERNANDES COSTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mateus Santana dos Santos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posto de Identificação Civil de Colatina(Linhares)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mikaely Freitas De Aquino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paloma Marçal Silva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yasmim Gomes Fernandes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YASMIN NERES SANTOS</t>
   </si>
 </sst>
 </file>
@@ -188,7 +263,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.7999"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -226,7 +301,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -239,15 +314,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -280,8 +359,8 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFBE3D6"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFBBE6FE"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF2A6099"/>
@@ -434,7 +513,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="53.14"/>
@@ -465,10 +544,10 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="3" t="n">
@@ -476,10 +555,10 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="3" t="n">
@@ -487,10 +566,10 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="3" t="n">
@@ -498,10 +577,10 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="3" t="n">
@@ -509,10 +588,10 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="3" t="n">
@@ -520,10 +599,10 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="3" t="n">
@@ -531,10 +610,10 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3" t="n">
@@ -542,10 +621,10 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
@@ -553,10 +632,10 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="3" t="n">
@@ -564,10 +643,10 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="3" t="n">
@@ -575,10 +654,10 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="3" t="n">
@@ -586,10 +665,10 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="3" t="n">
@@ -597,10 +676,10 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="3" t="n">
@@ -608,10 +687,10 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="3" t="n">
@@ -619,10 +698,10 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="3" t="n">
@@ -630,10 +709,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="3" t="n">
@@ -641,10 +720,10 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C19" s="3" t="n">
@@ -652,10 +731,10 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C20" s="3" t="n">
@@ -663,10 +742,10 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C21" s="3" t="n">
@@ -674,21 +753,21 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C22" s="6" t="n">
         <v>5170052</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C23" s="3" t="n">
@@ -696,14 +775,201 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C24" s="3" t="n">
         <v>5135524</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>5081912</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>5174465</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>5150256</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>5165571</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>5172870</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>5157129</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>5151120</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>5165326</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>5174430</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>5171300</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>5150442</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>5170001</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>5187133</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>5157188</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>5170877</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>5176182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>